<commit_message>
Refine D2 scientific validation figures
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/validation/D2_full_pipeline_injection_source_data.xlsx
+++ b/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/validation/D2_full_pipeline_injection_source_data.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T42"/>
+  <dimension ref="A1:T52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1806,7 +1806,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
         <v>46025.5</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>46025.52013888889</v>
+        <v>46025.51319444444</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1834,22 +1834,22 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>4.331944444444444</v>
+        <v>4.614814814814816</v>
       </c>
       <c r="L21" t="n">
-        <v>3.733333333333333</v>
+        <v>3.980808080808081</v>
       </c>
       <c r="M21" t="n">
         <v>5</v>
       </c>
       <c r="N21" t="n">
-        <v>4.213708333333333</v>
+        <v>4.399323232323232</v>
       </c>
       <c r="O21" t="n">
-        <v>30.4</v>
+        <v>24.46060606060606</v>
       </c>
       <c r="P21" t="n">
-        <v>18.87100000000001</v>
+        <v>14.41624242424244</v>
       </c>
       <c r="Q21" t="b">
         <v>1</v>
@@ -1861,7 +1861,7 @@
         <v>0</v>
       </c>
       <c r="T21" t="n">
-        <v>24.51666666666667</v>
+        <v>24.68333333333333</v>
       </c>
     </row>
     <row r="22">
@@ -1876,7 +1876,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1892,7 +1892,7 @@
         <v>46025.5</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>46025.54097222222</v>
+        <v>46025.52013888889</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1904,22 +1904,22 @@
         <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>3.880555555555556</v>
+        <v>4.331944444444444</v>
       </c>
       <c r="L22" t="n">
-        <v>3.3</v>
+        <v>3.733333333333333</v>
       </c>
       <c r="M22" t="n">
         <v>5</v>
       </c>
       <c r="N22" t="n">
-        <v>3.897916666666667</v>
+        <v>4.213708333333333</v>
       </c>
       <c r="O22" t="n">
-        <v>40.8</v>
+        <v>30.4</v>
       </c>
       <c r="P22" t="n">
-        <v>26.45</v>
+        <v>18.87100000000001</v>
       </c>
       <c r="Q22" t="b">
         <v>1</v>
@@ -1931,7 +1931,7 @@
         <v>0</v>
       </c>
       <c r="T22" t="n">
-        <v>24.01666666666667</v>
+        <v>24.51666666666667</v>
       </c>
     </row>
     <row r="23">
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>360</v>
+        <v>60</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
         <v>46025.5</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>46025.74930555555</v>
+        <v>46025.54097222222</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1974,28 +1974,28 @@
         <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>2.4</v>
+        <v>3.880555555555556</v>
       </c>
       <c r="L23" t="n">
-        <v>2.3</v>
+        <v>3.3</v>
       </c>
       <c r="M23" t="n">
         <v>5</v>
       </c>
       <c r="N23" t="n">
-        <v>1.8</v>
+        <v>3.897916666666667</v>
       </c>
       <c r="O23" t="n">
-        <v>70.80000000000003</v>
+        <v>40.8</v>
       </c>
       <c r="P23" t="n">
-        <v>81.60900000000001</v>
+        <v>26.45</v>
       </c>
       <c r="Q23" t="b">
         <v>1</v>
       </c>
       <c r="R23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
         <v>0</v>
@@ -2012,11 +2012,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ten_two_minute_gaps</t>
+          <t>single_gap_min</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>20</v>
+        <v>360</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
         <v>46025.5</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>46025.68819444445</v>
+        <v>46025.74930555555</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -2044,31 +2044,35 @@
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>4.614814814814816</v>
+        <v>2.4</v>
       </c>
       <c r="L24" t="n">
-        <v>4.7</v>
+        <v>2.3</v>
       </c>
       <c r="M24" t="n">
         <v>5</v>
       </c>
       <c r="N24" t="n">
-        <v>4.740555555555556</v>
+        <v>1.8</v>
       </c>
       <c r="O24" t="n">
-        <v>7.226666666666661</v>
+        <v>70.80000000000003</v>
       </c>
       <c r="P24" t="n">
-        <v>5.999377777777772</v>
+        <v>81.60900000000001</v>
       </c>
       <c r="Q24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R24" t="b">
-        <v>0</v>
-      </c>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" t="n">
+        <v>24.01666666666667</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2078,27 +2082,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>single_gap_min</t>
+          <t>ten_two_minute_gaps</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_1_1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ORP</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
         <v>46025.5</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>46025.50069444445</v>
+        <v>46025.68819444445</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -2110,22 +2114,22 @@
         <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>5</v>
+        <v>4.614814814814816</v>
       </c>
       <c r="L25" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="M25" t="n">
         <v>5</v>
       </c>
       <c r="N25" t="n">
-        <v>5</v>
+        <v>4.740555555555556</v>
       </c>
       <c r="O25" t="n">
-        <v>0</v>
+        <v>7.226666666666661</v>
       </c>
       <c r="P25" t="n">
-        <v>0</v>
+        <v>5.999377777777772</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2148,7 +2152,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2164,7 +2168,7 @@
         <v>46025.5</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>46025.50277777778</v>
+        <v>46025.50069444445</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -2179,19 +2183,19 @@
         <v>5</v>
       </c>
       <c r="L26" t="n">
-        <v>4.88</v>
+        <v>5</v>
       </c>
       <c r="M26" t="n">
         <v>5</v>
       </c>
       <c r="N26" t="n">
-        <v>4.938800000000001</v>
+        <v>5</v>
       </c>
       <c r="O26" t="n">
-        <v>2.880000000000003</v>
+        <v>0</v>
       </c>
       <c r="P26" t="n">
-        <v>1.468799999999987</v>
+        <v>0</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2214,7 +2218,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2230,7 +2234,7 @@
         <v>46025.5</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>46025.50347222222</v>
+        <v>46025.50277777778</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -2245,19 +2249,19 @@
         <v>5</v>
       </c>
       <c r="L27" t="n">
-        <v>4.77</v>
+        <v>4.88</v>
       </c>
       <c r="M27" t="n">
         <v>5</v>
       </c>
       <c r="N27" t="n">
-        <v>4.8827</v>
+        <v>4.938800000000001</v>
       </c>
       <c r="O27" t="n">
-        <v>5.519999999999989</v>
+        <v>2.880000000000003</v>
       </c>
       <c r="P27" t="n">
-        <v>2.815200000000004</v>
+        <v>1.468799999999987</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2280,7 +2284,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2296,7 +2300,7 @@
         <v>46025.5</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>46025.50972222222</v>
+        <v>46025.50347222222</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -2308,35 +2312,31 @@
         <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>4.765277777777778</v>
+        <v>5</v>
       </c>
       <c r="L28" t="n">
-        <v>4.104545454545454</v>
+        <v>4.77</v>
       </c>
       <c r="M28" t="n">
         <v>5</v>
       </c>
       <c r="N28" t="n">
-        <v>4.494026515151514</v>
+        <v>4.8827</v>
       </c>
       <c r="O28" t="n">
-        <v>21.49090909090909</v>
+        <v>5.519999999999989</v>
       </c>
       <c r="P28" t="n">
-        <v>12.14336363636366</v>
+        <v>2.815200000000004</v>
       </c>
       <c r="Q28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R28" t="b">
         <v>0</v>
       </c>
-      <c r="S28" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" t="n">
-        <v>24.76666666666667</v>
-      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2366,7 +2366,7 @@
         <v>46025.5</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>46025.52013888889</v>
+        <v>46025.50972222222</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -2378,22 +2378,22 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>4.331944444444444</v>
+        <v>4.765277777777778</v>
       </c>
       <c r="L29" t="n">
-        <v>3.733333333333333</v>
+        <v>4.104545454545454</v>
       </c>
       <c r="M29" t="n">
         <v>5</v>
       </c>
       <c r="N29" t="n">
-        <v>4.213708333333333</v>
+        <v>4.494026515151514</v>
       </c>
       <c r="O29" t="n">
-        <v>30.4</v>
+        <v>21.49090909090909</v>
       </c>
       <c r="P29" t="n">
-        <v>18.87100000000001</v>
+        <v>12.14336363636366</v>
       </c>
       <c r="Q29" t="b">
         <v>1</v>
@@ -2405,7 +2405,7 @@
         <v>0</v>
       </c>
       <c r="T29" t="n">
-        <v>24.51666666666667</v>
+        <v>24.76666666666667</v>
       </c>
     </row>
     <row r="30">
@@ -2420,7 +2420,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         <v>46025.5</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>46025.54097222222</v>
+        <v>46025.51319444444</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -2448,22 +2448,22 @@
         <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>3.880555555555556</v>
+        <v>4.614814814814816</v>
       </c>
       <c r="L30" t="n">
-        <v>3.3</v>
+        <v>3.980808080808081</v>
       </c>
       <c r="M30" t="n">
         <v>5</v>
       </c>
       <c r="N30" t="n">
-        <v>3.897916666666667</v>
+        <v>4.399323232323232</v>
       </c>
       <c r="O30" t="n">
-        <v>40.8</v>
+        <v>24.46060606060606</v>
       </c>
       <c r="P30" t="n">
-        <v>26.45</v>
+        <v>14.41624242424244</v>
       </c>
       <c r="Q30" t="b">
         <v>1</v>
@@ -2475,7 +2475,7 @@
         <v>0</v>
       </c>
       <c r="T30" t="n">
-        <v>24.01666666666667</v>
+        <v>24.68333333333333</v>
       </c>
     </row>
     <row r="31">
@@ -2490,7 +2490,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>360</v>
+        <v>30</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2506,7 +2506,7 @@
         <v>46025.5</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>46025.74930555555</v>
+        <v>46025.52013888889</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -2518,34 +2518,34 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>2.4</v>
+        <v>4.331944444444444</v>
       </c>
       <c r="L31" t="n">
-        <v>2.3</v>
+        <v>3.733333333333333</v>
       </c>
       <c r="M31" t="n">
         <v>5</v>
       </c>
       <c r="N31" t="n">
-        <v>1.8</v>
+        <v>4.213708333333333</v>
       </c>
       <c r="O31" t="n">
-        <v>70.80000000000003</v>
+        <v>30.4</v>
       </c>
       <c r="P31" t="n">
-        <v>81.60900000000001</v>
+        <v>18.87100000000001</v>
       </c>
       <c r="Q31" t="b">
         <v>1</v>
       </c>
       <c r="R31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S31" t="n">
         <v>0</v>
       </c>
       <c r="T31" t="n">
-        <v>24.01666666666667</v>
+        <v>24.51666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -2556,11 +2556,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ten_two_minute_gaps</t>
+          <t>single_gap_min</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2576,7 +2576,7 @@
         <v>46025.5</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>46025.68819444445</v>
+        <v>46025.54097222222</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -2588,61 +2588,65 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>4.614814814814816</v>
+        <v>3.880555555555556</v>
       </c>
       <c r="L32" t="n">
-        <v>4.7</v>
+        <v>3.3</v>
       </c>
       <c r="M32" t="n">
         <v>5</v>
       </c>
       <c r="N32" t="n">
-        <v>4.740555555555556</v>
+        <v>3.897916666666667</v>
       </c>
       <c r="O32" t="n">
-        <v>7.226666666666661</v>
+        <v>40.8</v>
       </c>
       <c r="P32" t="n">
-        <v>5.999377777777772</v>
+        <v>26.45</v>
       </c>
       <c r="Q32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R32" t="b">
         <v>0</v>
       </c>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
+      <c r="S32" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" t="n">
+        <v>24.01666666666667</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>stasis</t>
+          <t>gap</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>persistent_stasis_min</t>
+          <t>single_gap_min</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>10</v>
+        <v>360</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>DO_1_1</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>ORP</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
         <v>46025.5</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>46025.50625</v>
+        <v>46025.74930555555</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -2654,61 +2658,65 @@
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>5</v>
+        <v>2.4</v>
       </c>
       <c r="L33" t="n">
-        <v>5</v>
+        <v>2.3</v>
       </c>
       <c r="M33" t="n">
         <v>5</v>
       </c>
       <c r="N33" t="n">
-        <v>5</v>
+        <v>1.8</v>
       </c>
       <c r="O33" t="n">
-        <v>0</v>
+        <v>70.80000000000003</v>
       </c>
       <c r="P33" t="n">
-        <v>0</v>
+        <v>81.60900000000001</v>
       </c>
       <c r="Q33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R33" t="b">
-        <v>0</v>
-      </c>
-      <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" t="n">
+        <v>24.01666666666667</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>stasis</t>
+          <t>gap</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>persistent_stasis_min</t>
+          <t>ten_two_minute_gaps</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>DO_1_1</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>ORP</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
         <v>46025.5</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>46025.50972222222</v>
+        <v>46025.68819444445</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -2720,22 +2728,22 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>5</v>
+        <v>4.614814814814816</v>
       </c>
       <c r="L34" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="M34" t="n">
         <v>5</v>
       </c>
       <c r="N34" t="n">
-        <v>5</v>
+        <v>4.740555555555556</v>
       </c>
       <c r="O34" t="n">
-        <v>0</v>
+        <v>7.226666666666661</v>
       </c>
       <c r="P34" t="n">
-        <v>0</v>
+        <v>5.999377777777772</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2758,7 +2766,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2774,7 +2782,7 @@
         <v>46025.5</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>46025.51319444444</v>
+        <v>46025.50625</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -2824,7 +2832,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2840,7 +2848,7 @@
         <v>46025.5</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>46025.52013888889</v>
+        <v>46025.50972222222</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -2858,16 +2866,16 @@
         <v>5</v>
       </c>
       <c r="M36" t="n">
-        <v>4.638888888888889</v>
+        <v>5</v>
       </c>
       <c r="N36" t="n">
-        <v>4.790555555555557</v>
+        <v>5</v>
       </c>
       <c r="O36" t="n">
-        <v>2.166666666666664</v>
+        <v>0</v>
       </c>
       <c r="P36" t="n">
-        <v>1.256666666666661</v>
+        <v>0</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -2890,7 +2898,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2906,7 +2914,7 @@
         <v>46025.5</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>46025.54097222222</v>
+        <v>46025.51319444444</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -2924,29 +2932,25 @@
         <v>5</v>
       </c>
       <c r="M37" t="n">
-        <v>3.625</v>
+        <v>5</v>
       </c>
       <c r="N37" t="n">
-        <v>4.2025</v>
+        <v>5</v>
       </c>
       <c r="O37" t="n">
-        <v>8.25</v>
+        <v>0</v>
       </c>
       <c r="P37" t="n">
-        <v>4.785000000000002</v>
+        <v>0</v>
       </c>
       <c r="Q37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R37" t="b">
         <v>0</v>
       </c>
-      <c r="S37" t="n">
-        <v>0</v>
-      </c>
-      <c r="T37" t="n">
-        <v>6.016666666666667</v>
-      </c>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2960,23 +2964,23 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_1_1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ORP</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
         <v>46025.5</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>46025.50625</v>
+        <v>46025.52013888889</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -2994,16 +2998,16 @@
         <v>5</v>
       </c>
       <c r="M38" t="n">
-        <v>5</v>
+        <v>4.638888888888889</v>
       </c>
       <c r="N38" t="n">
-        <v>5</v>
+        <v>4.790555555555557</v>
       </c>
       <c r="O38" t="n">
-        <v>0</v>
+        <v>2.166666666666664</v>
       </c>
       <c r="P38" t="n">
-        <v>0</v>
+        <v>1.256666666666661</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3026,23 +3030,23 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_1_1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ORP</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
         <v>46025.5</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>46025.50972222222</v>
+        <v>46025.53055555555</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -3060,25 +3064,29 @@
         <v>5</v>
       </c>
       <c r="M39" t="n">
-        <v>5</v>
+        <v>3.972222222222222</v>
       </c>
       <c r="N39" t="n">
-        <v>5</v>
+        <v>4.403888888888888</v>
       </c>
       <c r="O39" t="n">
-        <v>0</v>
+        <v>6.166666666666666</v>
       </c>
       <c r="P39" t="n">
-        <v>0</v>
+        <v>3.576666666666672</v>
       </c>
       <c r="Q39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R39" t="b">
         <v>0</v>
       </c>
-      <c r="S39" t="inlineStr"/>
-      <c r="T39" t="inlineStr"/>
+      <c r="S39" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" t="n">
+        <v>6.266666666666667</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3092,23 +3100,23 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_1_1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ORP</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
         <v>46025.5</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>46025.51319444444</v>
+        <v>46025.54097222222</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -3126,25 +3134,29 @@
         <v>5</v>
       </c>
       <c r="M40" t="n">
-        <v>5</v>
+        <v>3.625</v>
       </c>
       <c r="N40" t="n">
-        <v>5</v>
+        <v>4.2025</v>
       </c>
       <c r="O40" t="n">
-        <v>0</v>
+        <v>8.25</v>
       </c>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>4.785000000000002</v>
       </c>
       <c r="Q40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R40" t="b">
         <v>0</v>
       </c>
-      <c r="S40" t="inlineStr"/>
-      <c r="T40" t="inlineStr"/>
+      <c r="S40" t="n">
+        <v>0</v>
+      </c>
+      <c r="T40" t="n">
+        <v>6.016666666666667</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3158,23 +3170,23 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_1_1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ORP</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
         <v>46025.5</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>46025.52013888889</v>
+        <v>46025.56180555555</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -3192,25 +3204,29 @@
         <v>5</v>
       </c>
       <c r="M41" t="n">
-        <v>4.638888888888889</v>
+        <v>2.972222222222222</v>
       </c>
       <c r="N41" t="n">
-        <v>4.790555555555557</v>
+        <v>3.823888888888889</v>
       </c>
       <c r="O41" t="n">
-        <v>2.166666666666664</v>
+        <v>12.54166666666667</v>
       </c>
       <c r="P41" t="n">
-        <v>1.256666666666661</v>
+        <v>7.274166666666668</v>
       </c>
       <c r="Q41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R41" t="b">
         <v>0</v>
       </c>
-      <c r="S41" t="inlineStr"/>
-      <c r="T41" t="inlineStr"/>
+      <c r="S41" t="n">
+        <v>0</v>
+      </c>
+      <c r="T41" t="n">
+        <v>6.516666666666667</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3224,23 +3240,23 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_1_1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ORP</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
         <v>46025.5</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>46025.54097222222</v>
+        <v>46025.58263888889</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -3258,16 +3274,16 @@
         <v>5</v>
       </c>
       <c r="M42" t="n">
-        <v>3.625</v>
+        <v>2.694444444444445</v>
       </c>
       <c r="N42" t="n">
-        <v>4.2025</v>
+        <v>3.662777777777777</v>
       </c>
       <c r="O42" t="n">
-        <v>8.25</v>
+        <v>14.625</v>
       </c>
       <c r="P42" t="n">
-        <v>4.785000000000002</v>
+        <v>8.482500000000002</v>
       </c>
       <c r="Q42" t="b">
         <v>1</v>
@@ -3279,6 +3295,690 @@
         <v>0</v>
       </c>
       <c r="T42" t="n">
+        <v>6.016666666666667</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>stasis</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>persistent_stasis_min</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>180</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>DO_1_1</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>46025.5</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>46025.62430555555</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="n">
+        <v>5</v>
+      </c>
+      <c r="L43" t="n">
+        <v>5</v>
+      </c>
+      <c r="M43" t="n">
+        <v>2.138888888888889</v>
+      </c>
+      <c r="N43" t="n">
+        <v>3.340555555555556</v>
+      </c>
+      <c r="O43" t="n">
+        <v>19.29166666666667</v>
+      </c>
+      <c r="P43" t="n">
+        <v>11.18916666666667</v>
+      </c>
+      <c r="Q43" t="b">
+        <v>1</v>
+      </c>
+      <c r="R43" t="b">
+        <v>0</v>
+      </c>
+      <c r="S43" t="n">
+        <v>0</v>
+      </c>
+      <c r="T43" t="n">
+        <v>6.016666666666667</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>stasis</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>persistent_stasis_min</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>10</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ORP_1_1</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>46025.5</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>46025.50625</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>5</v>
+      </c>
+      <c r="L44" t="n">
+        <v>5</v>
+      </c>
+      <c r="M44" t="n">
+        <v>5</v>
+      </c>
+      <c r="N44" t="n">
+        <v>5</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="b">
+        <v>0</v>
+      </c>
+      <c r="R44" t="b">
+        <v>0</v>
+      </c>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>stasis</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>persistent_stasis_min</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>15</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>ORP_1_1</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>46025.5</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>46025.50972222222</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>5</v>
+      </c>
+      <c r="L45" t="n">
+        <v>5</v>
+      </c>
+      <c r="M45" t="n">
+        <v>5</v>
+      </c>
+      <c r="N45" t="n">
+        <v>5</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="b">
+        <v>0</v>
+      </c>
+      <c r="R45" t="b">
+        <v>0</v>
+      </c>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>stasis</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>persistent_stasis_min</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>20</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ORP_1_1</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>46025.5</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>46025.51319444444</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>5</v>
+      </c>
+      <c r="L46" t="n">
+        <v>5</v>
+      </c>
+      <c r="M46" t="n">
+        <v>5</v>
+      </c>
+      <c r="N46" t="n">
+        <v>5</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" t="b">
+        <v>0</v>
+      </c>
+      <c r="R46" t="b">
+        <v>0</v>
+      </c>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>stasis</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>persistent_stasis_min</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>30</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ORP_1_1</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>46025.5</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>46025.52013888889</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>5</v>
+      </c>
+      <c r="L47" t="n">
+        <v>5</v>
+      </c>
+      <c r="M47" t="n">
+        <v>4.638888888888889</v>
+      </c>
+      <c r="N47" t="n">
+        <v>4.790555555555557</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2.166666666666664</v>
+      </c>
+      <c r="P47" t="n">
+        <v>1.256666666666661</v>
+      </c>
+      <c r="Q47" t="b">
+        <v>0</v>
+      </c>
+      <c r="R47" t="b">
+        <v>0</v>
+      </c>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>stasis</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>persistent_stasis_min</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>45</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ORP_1_1</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>46025.5</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>46025.53055555555</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>5</v>
+      </c>
+      <c r="L48" t="n">
+        <v>5</v>
+      </c>
+      <c r="M48" t="n">
+        <v>3.972222222222222</v>
+      </c>
+      <c r="N48" t="n">
+        <v>4.403888888888888</v>
+      </c>
+      <c r="O48" t="n">
+        <v>6.166666666666666</v>
+      </c>
+      <c r="P48" t="n">
+        <v>3.576666666666672</v>
+      </c>
+      <c r="Q48" t="b">
+        <v>1</v>
+      </c>
+      <c r="R48" t="b">
+        <v>0</v>
+      </c>
+      <c r="S48" t="n">
+        <v>0</v>
+      </c>
+      <c r="T48" t="n">
+        <v>6.266666666666667</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>stasis</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>persistent_stasis_min</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>60</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ORP_1_1</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>46025.5</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>46025.54097222222</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="n">
+        <v>5</v>
+      </c>
+      <c r="L49" t="n">
+        <v>5</v>
+      </c>
+      <c r="M49" t="n">
+        <v>3.625</v>
+      </c>
+      <c r="N49" t="n">
+        <v>4.2025</v>
+      </c>
+      <c r="O49" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="P49" t="n">
+        <v>4.785000000000002</v>
+      </c>
+      <c r="Q49" t="b">
+        <v>1</v>
+      </c>
+      <c r="R49" t="b">
+        <v>0</v>
+      </c>
+      <c r="S49" t="n">
+        <v>0</v>
+      </c>
+      <c r="T49" t="n">
+        <v>6.016666666666667</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>stasis</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>persistent_stasis_min</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>90</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ORP_1_1</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>46025.5</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>46025.56180555555</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" t="n">
+        <v>5</v>
+      </c>
+      <c r="L50" t="n">
+        <v>5</v>
+      </c>
+      <c r="M50" t="n">
+        <v>2.972222222222222</v>
+      </c>
+      <c r="N50" t="n">
+        <v>3.823888888888889</v>
+      </c>
+      <c r="O50" t="n">
+        <v>12.54166666666667</v>
+      </c>
+      <c r="P50" t="n">
+        <v>7.274166666666668</v>
+      </c>
+      <c r="Q50" t="b">
+        <v>1</v>
+      </c>
+      <c r="R50" t="b">
+        <v>0</v>
+      </c>
+      <c r="S50" t="n">
+        <v>0</v>
+      </c>
+      <c r="T50" t="n">
+        <v>6.516666666666667</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>stasis</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>persistent_stasis_min</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>120</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ORP_1_1</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>46025.5</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>46025.58263888889</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="n">
+        <v>5</v>
+      </c>
+      <c r="L51" t="n">
+        <v>5</v>
+      </c>
+      <c r="M51" t="n">
+        <v>2.694444444444445</v>
+      </c>
+      <c r="N51" t="n">
+        <v>3.662777777777777</v>
+      </c>
+      <c r="O51" t="n">
+        <v>14.625</v>
+      </c>
+      <c r="P51" t="n">
+        <v>8.482500000000002</v>
+      </c>
+      <c r="Q51" t="b">
+        <v>1</v>
+      </c>
+      <c r="R51" t="b">
+        <v>0</v>
+      </c>
+      <c r="S51" t="n">
+        <v>0</v>
+      </c>
+      <c r="T51" t="n">
+        <v>6.016666666666667</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>stasis</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>persistent_stasis_min</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>180</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ORP_1_1</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>46025.5</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>46025.62430555555</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M52" t="n">
+        <v>2.138888888888889</v>
+      </c>
+      <c r="N52" t="n">
+        <v>3.340555555555556</v>
+      </c>
+      <c r="O52" t="n">
+        <v>19.29166666666667</v>
+      </c>
+      <c r="P52" t="n">
+        <v>11.18916666666667</v>
+      </c>
+      <c r="Q52" t="b">
+        <v>1</v>
+      </c>
+      <c r="R52" t="b">
+        <v>0</v>
+      </c>
+      <c r="S52" t="n">
+        <v>0</v>
+      </c>
+      <c r="T52" t="n">
         <v>6.016666666666667</v>
       </c>
     </row>
@@ -5895,7 +6595,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -5921,7 +6621,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -5947,10 +6647,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8944271909999157</v>
+        <v>0.9831920802501751</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -5973,10 +6673,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8944271909999157</v>
+        <v>0.9831920802501751</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>

</xml_diff>